<commit_message>
Update chip report site 2026-08-13
</commit_message>
<xml_diff>
--- a/outputs/chip-report/台股盤後籌碼_2026-06-18.xlsx
+++ b/outputs/chip-report/台股盤後籌碼_2026-06-18.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N114"/>
+  <dimension ref="A1:N126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -582,7 +582,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>本次為 2026-06-18 正式版，已補入 TWSE 與 TAIFEX 官方數據；加權指數當日高低差使用 TWSE MI_5MINS_HIST 官方資料，散戶與微台欄位沿用全市場 OI 減三大法人多空單的原表邏輯回推。</t>
+          <t>本次為 2026-06-18 正式版，已補入 TWSE 與 TAIFEX 官方數據；散戶位階採 45 日中位秩分位，並以小台部位 + 微台部位/5 換算等值口數。</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       <c r="F40" s="6" t="n"/>
       <c r="G40" s="6" t="n"/>
       <c r="I40" s="6" t="n">
-        <v>-197</v>
+        <v>197</v>
       </c>
       <c r="J40" s="6" t="n"/>
       <c r="K40" s="6" t="n"/>
@@ -1094,7 +1094,7 @@
       <c r="G42" s="7" t="n"/>
       <c r="I42" s="7" t="inlineStr">
         <is>
-          <t>|-67,652.85| - |-67,850| ≈ -197；結算日基準 6/17；結算後首日，本欄基準為昨日結算日 6/17。</t>
+          <t>-67,652.85 - (-67,850) ≈ 197；結算日基準 6/17；結算後首日，本欄基準為昨日結算日 6/17。</t>
         </is>
       </c>
       <c r="J42" s="7" t="n"/>
@@ -1888,6 +1888,13 @@
       </c>
       <c r="F103" s="15" t="n"/>
       <c r="G103" s="15" t="n"/>
+      <c r="I103" s="15" t="inlineStr">
+        <is>
+          <t>小台+微台等值多單</t>
+        </is>
+      </c>
+      <c r="J103" s="15" t="n"/>
+      <c r="K103" s="15" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="6" t="n">
@@ -1900,6 +1907,11 @@
       </c>
       <c r="F104" s="6" t="n"/>
       <c r="G104" s="6" t="n"/>
+      <c r="I104" s="6" t="n">
+        <v>38210.6</v>
+      </c>
+      <c r="J104" s="6" t="n"/>
+      <c r="K104" s="6" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="6" t="n"/>
@@ -1908,6 +1920,9 @@
       <c r="E105" s="6" t="n"/>
       <c r="F105" s="6" t="n"/>
       <c r="G105" s="6" t="n"/>
+      <c r="I105" s="6" t="n"/>
+      <c r="J105" s="6" t="n"/>
+      <c r="K105" s="6" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="7" t="inlineStr">
@@ -1924,6 +1939,13 @@
       </c>
       <c r="F106" s="7" t="n"/>
       <c r="G106" s="7" t="n"/>
+      <c r="I106" s="7" t="inlineStr">
+        <is>
+          <t>28,106 + 50,523 / 5；微台 5 口換算 1 口小台等值</t>
+        </is>
+      </c>
+      <c r="J106" s="7" t="n"/>
+      <c r="K106" s="7" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="7" t="n"/>
@@ -1932,23 +1954,199 @@
       <c r="E107" s="7" t="n"/>
       <c r="F107" s="7" t="n"/>
       <c r="G107" s="7" t="n"/>
+      <c r="I107" s="7" t="n"/>
+      <c r="J107" s="7" t="n"/>
+      <c r="K107" s="7" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="15" t="inlineStr">
+        <is>
+          <t>小台+微台等值空單</t>
+        </is>
+      </c>
+      <c r="B109" s="15" t="n"/>
+      <c r="C109" s="15" t="n"/>
+      <c r="E109" s="15" t="inlineStr">
+        <is>
+          <t>小台+微台等值淨多空</t>
+        </is>
+      </c>
+      <c r="F109" s="15" t="n"/>
+      <c r="G109" s="15" t="n"/>
+      <c r="I109" s="15" t="inlineStr">
+        <is>
+          <t>散戶多方位階(45日)</t>
+        </is>
+      </c>
+      <c r="J109" s="15" t="n"/>
+      <c r="K109" s="15" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="16" t="inlineStr">
-        <is>
-          <t>這是 2026-06-18 的盤後籌碼正式版：加權指數收 46,465.20 點、漲 587.81 點，盤中最高 46,565.70 點、最低 45,972.26 點，成交值約 16,061.95 億元；TWSE 信用交易統計已補回，融資金額餘額 5,930.47 億、較前一交易日增加 82.86 億，融券餘額 204,357 張、較前一交易日增加 12,318 張。TAIFEX 的外資(大小台)期貨未平倉依原表合併口徑 = TXF + MXF/4 + TMF/20，6/18 約為 -67,653，與結算比約 -197、與前日增減約 197；主表 OP 欄位維持 BC-SC 與 BP-SP 的淨額口徑。</t>
-        </is>
-      </c>
-    </row>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
+      <c r="A110" s="6" t="n">
+        <v>30074.8</v>
+      </c>
+      <c r="B110" s="6" t="n"/>
+      <c r="C110" s="6" t="n"/>
+      <c r="E110" s="6" t="n">
+        <v>8135.799999999999</v>
+      </c>
+      <c r="F110" s="6" t="n"/>
+      <c r="G110" s="6" t="n"/>
+      <c r="I110" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="J110" s="6" t="n"/>
+      <c r="K110" s="6" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="6" t="n"/>
+      <c r="B111" s="6" t="n"/>
+      <c r="C111" s="6" t="n"/>
+      <c r="E111" s="6" t="n"/>
+      <c r="F111" s="6" t="n"/>
+      <c r="G111" s="6" t="n"/>
+      <c r="I111" s="6" t="n"/>
+      <c r="J111" s="6" t="n"/>
+      <c r="K111" s="6" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="7" t="inlineStr">
+        <is>
+          <t>22,434 + 38,204 / 5；微台 5 口換算 1 口小台等值</t>
+        </is>
+      </c>
+      <c r="B112" s="7" t="n"/>
+      <c r="C112" s="7" t="n"/>
+      <c r="E112" s="7" t="inlineStr">
+        <is>
+          <t>38,210.6 - 30,074.8</t>
+        </is>
+      </c>
+      <c r="F112" s="7" t="n"/>
+      <c r="G112" s="7" t="n"/>
+      <c r="I112" s="7" t="inlineStr">
+        <is>
+          <t>中位秩百分位 = (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 41 筆。</t>
+        </is>
+      </c>
+      <c r="J112" s="7" t="n"/>
+      <c r="K112" s="7" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="7" t="n"/>
+      <c r="B113" s="7" t="n"/>
+      <c r="C113" s="7" t="n"/>
+      <c r="E113" s="7" t="n"/>
+      <c r="F113" s="7" t="n"/>
+      <c r="G113" s="7" t="n"/>
+      <c r="I113" s="7" t="n"/>
+      <c r="J113" s="7" t="n"/>
+      <c r="K113" s="7" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="15" t="inlineStr">
+        <is>
+          <t>散戶空方位階(45日)</t>
+        </is>
+      </c>
+      <c r="B115" s="15" t="n"/>
+      <c r="C115" s="15" t="n"/>
+      <c r="E115" s="15" t="inlineStr">
+        <is>
+          <t>散戶淨多空位階(45日)</t>
+        </is>
+      </c>
+      <c r="F115" s="15" t="n"/>
+      <c r="G115" s="15" t="n"/>
+      <c r="I115" s="15" t="inlineStr">
+        <is>
+          <t>微台多空比位階(45日)</t>
+        </is>
+      </c>
+      <c r="J115" s="15" t="n"/>
+      <c r="K115" s="15" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B116" s="6" t="n"/>
+      <c r="C116" s="6" t="n"/>
+      <c r="E116" s="6" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="F116" s="6" t="n"/>
+      <c r="G116" s="6" t="n"/>
+      <c r="I116" s="6" t="n">
+        <v>45.1</v>
+      </c>
+      <c r="J116" s="6" t="n"/>
+      <c r="K116" s="6" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="6" t="n"/>
+      <c r="B117" s="6" t="n"/>
+      <c r="C117" s="6" t="n"/>
+      <c r="E117" s="6" t="n"/>
+      <c r="F117" s="6" t="n"/>
+      <c r="G117" s="6" t="n"/>
+      <c r="I117" s="6" t="n"/>
+      <c r="J117" s="6" t="n"/>
+      <c r="K117" s="6" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="7" t="inlineStr">
+        <is>
+          <t>中位秩百分位 = (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 41 筆。</t>
+        </is>
+      </c>
+      <c r="B118" s="7" t="n"/>
+      <c r="C118" s="7" t="n"/>
+      <c r="E118" s="7" t="inlineStr">
+        <is>
+          <t>中位秩百分位 = (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 41 筆。</t>
+        </is>
+      </c>
+      <c r="F118" s="7" t="n"/>
+      <c r="G118" s="7" t="n"/>
+      <c r="I118" s="7" t="inlineStr">
+        <is>
+          <t>中位秩百分位 = (低於本日筆數 + 同值筆數 / 2) / 樣本數 x 100。 小台＋微台等值口數；微台 5 口換算為 1 口小台等值。；目前樣本 41 筆。</t>
+        </is>
+      </c>
+      <c r="J118" s="7" t="n"/>
+      <c r="K118" s="7" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="7" t="n"/>
+      <c r="B119" s="7" t="n"/>
+      <c r="C119" s="7" t="n"/>
+      <c r="E119" s="7" t="n"/>
+      <c r="F119" s="7" t="n"/>
+      <c r="G119" s="7" t="n"/>
+      <c r="I119" s="7" t="n"/>
+      <c r="J119" s="7" t="n"/>
+      <c r="K119" s="7" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="16" t="inlineStr">
+        <is>
+          <t>這是 2026-06-18 的盤後籌碼正式版：加權指數收 46,465.20 點、漲 587.81 點，盤中最高 46,565.70 點、最低 45,972.26 點，成交值約 16,061.95 億元；TWSE 信用交易統計已補回，融資金額餘額 5,930.47 億、較前一交易日增加 82.86 億，融券餘額 204,357 張、較前一交易日增加 12,318 張。TAIFEX 的外資(大小台)期貨未平倉依原表合併口徑 = TXF + MXF/4 + TMF/20，6/18 約為 -67,653，與結算比約 197、與前日增減約 197；主表 OP 欄位維持 BC-SC 與 BP-SP 的淨額口徑。</t>
+        </is>
+      </c>
+    </row>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
   </sheetData>
-  <mergeCells count="137">
+  <mergeCells count="158">
+    <mergeCell ref="E116:G117"/>
+    <mergeCell ref="I103:K103"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="E72:G73"/>
     <mergeCell ref="I97:K97"/>
+    <mergeCell ref="I110:K111"/>
     <mergeCell ref="A34:C35"/>
     <mergeCell ref="A57:C57"/>
     <mergeCell ref="A71:C71"/>
@@ -1960,8 +2158,10 @@
     <mergeCell ref="E57:G57"/>
     <mergeCell ref="E48:G49"/>
     <mergeCell ref="A91:C91"/>
+    <mergeCell ref="I104:K105"/>
     <mergeCell ref="A16:C17"/>
     <mergeCell ref="I26:K27"/>
+    <mergeCell ref="I106:K107"/>
     <mergeCell ref="I65:K65"/>
     <mergeCell ref="A77:C77"/>
     <mergeCell ref="E74:G75"/>
@@ -1973,9 +2173,11 @@
     <mergeCell ref="A22:C23"/>
     <mergeCell ref="I42:K43"/>
     <mergeCell ref="I20:K21"/>
+    <mergeCell ref="A116:C117"/>
     <mergeCell ref="I60:K61"/>
     <mergeCell ref="A20:C21"/>
     <mergeCell ref="A72:C73"/>
+    <mergeCell ref="I115:K115"/>
     <mergeCell ref="E100:G101"/>
     <mergeCell ref="A28:C29"/>
     <mergeCell ref="A1:N1"/>
@@ -1983,10 +2185,10 @@
     <mergeCell ref="E22:G23"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="E14:G15"/>
+    <mergeCell ref="A110:C111"/>
     <mergeCell ref="A48:C49"/>
     <mergeCell ref="A97:C97"/>
     <mergeCell ref="E78:G79"/>
-    <mergeCell ref="A110:N114"/>
     <mergeCell ref="I51:K51"/>
     <mergeCell ref="A54:C55"/>
     <mergeCell ref="I72:K73"/>
@@ -1995,10 +2197,12 @@
     <mergeCell ref="E97:G97"/>
     <mergeCell ref="A12:N12"/>
     <mergeCell ref="A31:C31"/>
+    <mergeCell ref="E109:G109"/>
     <mergeCell ref="A74:C75"/>
     <mergeCell ref="A46:C47"/>
     <mergeCell ref="A51:C51"/>
     <mergeCell ref="E71:G71"/>
+    <mergeCell ref="I112:K113"/>
     <mergeCell ref="E46:G47"/>
     <mergeCell ref="E40:G41"/>
     <mergeCell ref="A4:N4"/>
@@ -2010,6 +2214,7 @@
     <mergeCell ref="I25:K25"/>
     <mergeCell ref="I98:K99"/>
     <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A122:N126"/>
     <mergeCell ref="E19:G19"/>
     <mergeCell ref="E26:G27"/>
     <mergeCell ref="A68:C69"/>
@@ -2031,10 +2236,15 @@
     <mergeCell ref="A78:C79"/>
     <mergeCell ref="E60:G61"/>
     <mergeCell ref="A6:C7"/>
+    <mergeCell ref="I109:K109"/>
+    <mergeCell ref="I116:K117"/>
+    <mergeCell ref="E115:G115"/>
     <mergeCell ref="I13:K13"/>
     <mergeCell ref="A80:C81"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="I100:K101"/>
+    <mergeCell ref="E118:G119"/>
+    <mergeCell ref="I118:K119"/>
     <mergeCell ref="E28:G29"/>
     <mergeCell ref="E94:G95"/>
     <mergeCell ref="A26:C27"/>
@@ -2046,26 +2256,31 @@
     <mergeCell ref="E51:G51"/>
     <mergeCell ref="E16:G17"/>
     <mergeCell ref="I94:K95"/>
+    <mergeCell ref="A112:C113"/>
     <mergeCell ref="A106:C107"/>
     <mergeCell ref="A64:N64"/>
     <mergeCell ref="I71:K71"/>
     <mergeCell ref="I74:K75"/>
+    <mergeCell ref="E112:G113"/>
     <mergeCell ref="A58:C59"/>
     <mergeCell ref="I80:K81"/>
     <mergeCell ref="A40:C41"/>
     <mergeCell ref="A98:C99"/>
     <mergeCell ref="A90:N90"/>
     <mergeCell ref="A60:C61"/>
+    <mergeCell ref="A109:C109"/>
     <mergeCell ref="I66:K67"/>
     <mergeCell ref="E91:G91"/>
     <mergeCell ref="E25:G25"/>
     <mergeCell ref="E98:G99"/>
     <mergeCell ref="E20:G21"/>
     <mergeCell ref="I19:K19"/>
+    <mergeCell ref="A115:C115"/>
     <mergeCell ref="A19:C19"/>
     <mergeCell ref="A66:C67"/>
     <mergeCell ref="I22:K23"/>
     <mergeCell ref="I28:K29"/>
+    <mergeCell ref="A118:C119"/>
     <mergeCell ref="A39:C39"/>
     <mergeCell ref="I52:K53"/>
     <mergeCell ref="I92:K93"/>
@@ -2078,6 +2293,7 @@
     <mergeCell ref="A32:C33"/>
     <mergeCell ref="E39:G39"/>
     <mergeCell ref="A14:C15"/>
+    <mergeCell ref="E110:G111"/>
     <mergeCell ref="A42:C43"/>
     <mergeCell ref="A100:C101"/>
     <mergeCell ref="A65:C65"/>

</xml_diff>